<commit_message>
feat: enrich Excel execution report
</commit_message>
<xml_diff>
--- a/reports/sample-execution-report.xlsx
+++ b/reports/sample-execution-report.xlsx
@@ -11,54 +11,88 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
   <si>
     <t>Test Case ID</t>
   </si>
   <si>
-    <t>Title</t>
+    <t>Test Case Title</t>
   </si>
   <si>
     <t>Priority</t>
   </si>
   <si>
+    <t>Business Rationale</t>
+  </si>
+  <si>
     <t>Preconditions</t>
   </si>
   <si>
+    <t>Test Data</t>
+  </si>
+  <si>
     <t>Steps</t>
   </si>
   <si>
     <t>Expected Result</t>
   </si>
   <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Screenshot</t>
+  </si>
+  <si>
     <t>Error</t>
   </si>
   <si>
     <t>TC-01</t>
   </si>
   <si>
-    <t>Search for a product and verify product details</t>
+    <t>Search for a product, select a product and verify product details</t>
   </si>
   <si>
     <t>P0</t>
   </si>
   <si>
-    <t>Amazon.in is reachable and search results are available.</t>
-  </si>
-  <si>
-    <t>Open Amazon, search for the configured keyword, open a visible product result, and inspect its details.</t>
-  </si>
-  <si>
-    <t>A product page opens with a title, price, and availability information.</t>
+    <t>Product discovery and accurate product information are essential for customers to make purchase decisions.</t>
+  </si>
+  <si>
+    <t>Amazon.in is reachable, and a relevant product is available.</t>
+  </si>
+  <si>
+    <t>Configured search keyword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Amazon.in.
+2. Search for the product.
+3. Verify relevant search results.
+4. Open a product.
+5. Verify its title, price, and availability information.</t>
+  </si>
+  <si>
+    <t>Relevant search results appear, a product can be selected, the product page opens, and expected product information is displayed.</t>
+  </si>
+  <si>
+    <t>Product page opened and product details were visible.</t>
   </si>
   <si>
     <t>Pass</t>
   </si>
   <si>
-    <t/>
+    <t>Search phrase: wireless keyboard; Product title: HP K270 Wireless Keyboard; Price: ₹499.00; Availability: In stock</t>
+  </si>
+  <si>
+    <t>See embedded image</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
   <si>
     <t>TC-02</t>
@@ -67,25 +101,51 @@
     <t>Add a product to the cart</t>
   </si>
   <si>
-    <t>A purchasable product is available for the configured keyword.</t>
-  </si>
-  <si>
-    <t>Search, open a product, and add it to the cart.</t>
-  </si>
-  <si>
-    <t>Amazon confirms that the product was added.</t>
+    <t>Adding an item to the cart is a core step in the purchase journey.</t>
+  </si>
+  <si>
+    <t>Amazon.in is reachable, and a purchasable product is available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for a product.
+2. Open its product details page.
+3. Click Add to Cart.
+4. Verify the cart confirmation.</t>
+  </si>
+  <si>
+    <t>The selected product is added to the cart, and an appropriate confirmation is displayed.</t>
+  </si>
+  <si>
+    <t>Product was added to the cart and Amazon displayed a confirmation.</t>
+  </si>
+  <si>
+    <t>Search phrase: wireless keyboard; Product title: HP K270 Wireless Keyboard; Price: ₹499.00; Availability: In stock; Cart confirmation: displayed</t>
   </si>
   <si>
     <t>TC-03</t>
   </si>
   <si>
-    <t>Verify the cart contains the selected product</t>
-  </si>
-  <si>
-    <t>Search, open a product, add it to the cart, and open the cart.</t>
-  </si>
-  <si>
-    <t>The cart contains the selected product ASIN.</t>
+    <t>Verify cart contents</t>
+  </si>
+  <si>
+    <t>Customers need confidence that their cart contains the intended product before checkout.</t>
+  </si>
+  <si>
+    <t>The test establishes its own cart state by adding a product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for and add the product.
+2. Open the cart.
+3. Verify the selected product identity.</t>
+  </si>
+  <si>
+    <t>The intended product appears in the cart with quantity 1.</t>
+  </si>
+  <si>
+    <t>Selected product was found in the cart with quantity 1.</t>
+  </si>
+  <si>
+    <t>Search phrase: wireless keyboard; Product title: HP K270 Wireless Keyboard; Price: ₹499.00; Availability: In stock; Selected ASIN: B0DXPHFMLX; Quantity: 1</t>
   </si>
   <si>
     <t>TC-04</t>
@@ -94,10 +154,23 @@
     <t>Update cart quantity from 1 to 2</t>
   </si>
   <si>
-    <t>Add a product to the cart and increase its quantity.</t>
-  </si>
-  <si>
-    <t>The selected cart item quantity updates from 1 to 2.</t>
+    <t>Customers need to update the quantity of an item in their cart before checkout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for and select a product.
+2. Add it to the cart.
+3. Verify initial quantity 1.
+4. Increase the quantity to 2.
+5. Verify displayed quantity 2.</t>
+  </si>
+  <si>
+    <t>The selected product quantity changes from 1 to 2 and the cart displays the updated quantity.</t>
+  </si>
+  <si>
+    <t>Selected product quantity successfully changed from 1 to 2.</t>
+  </si>
+  <si>
+    <t>Search phrase: wireless keyboard; Product title: HP K270 Wireless Keyboard; Price: ₹499.00; Availability: In stock; Initial quantity: 1; Final quantity: 2</t>
   </si>
   <si>
     <t>TC-05</t>
@@ -106,17 +179,33 @@
     <t>Proceed from cart to checkout</t>
   </si>
   <si>
-    <t>Add a product to the cart and select Proceed to Buy.</t>
-  </si>
-  <si>
-    <t>Amazon reaches the sign-in boundary; no order or payment is attempted.</t>
+    <t>Checkout is a critical stage in the purchase journey; a blocker can prevent customers from completing purchases.</t>
+  </si>
+  <si>
+    <t>The test establishes its own cart state by adding a purchasable product. The browser should be signed out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Search for and select a product.
+2. Add it to the cart and open the cart.
+3. Select Proceed to Buy.
+4. Verify the sign-in requirement.
+5. Stop before placing an order or submitting payment.</t>
+  </si>
+  <si>
+    <t>The checkout journey advances to a sign-in requirement. No order or payment is submitted.</t>
+  </si>
+  <si>
+    <t>Amazon displayed the sign-in requirement. The test stopped before placing an order or payment.</t>
+  </si>
+  <si>
+    <t>Search phrase: wireless keyboard; Product title: HP K270 Wireless Keyboard; Price: ₹499.00; Availability: In stock; Checkout outcome: sign-in requirement displayed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -127,6 +216,11 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF006100"/>
     </font>
   </fonts>
   <fills count="4">
@@ -147,7 +241,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -155,18 +249,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -183,6 +300,206 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="857250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="857250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="857250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="857250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="857250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -507,177 +824,271 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
-    <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="8" width="32" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="32" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
+    <row r="2" ht="105" customHeight="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="D2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
+    <row r="3" ht="105" customHeight="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2" t="s">
+      <c r="G3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" ht="105" customHeight="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="D4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="5" ht="105" customHeight="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="K5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" ht="105" customHeight="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="M6" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>